<commit_message>
new method in preprocessing : L1 Normalisation : Least Absolute Deviation
</commit_message>
<xml_diff>
--- a/Excel/004 Data Processing.xlsx
+++ b/Excel/004 Data Processing.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{004BDF32-7D5B-46F5-A987-BF29759376E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CD19F8-7A53-44C2-9894-5D56AD83F997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binarisation" sheetId="1" r:id="rId1"/>
     <sheet name="Scalling" sheetId="2" r:id="rId2"/>
+    <sheet name="Normalisation (L1)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
   <si>
     <t>sample_data</t>
   </si>
@@ -51,12 +52,21 @@
   <si>
     <t>Selisih</t>
   </si>
+  <si>
+    <t>Least Absolute Deviations</t>
+  </si>
+  <si>
+    <t>Total Absolut Baris (L1 Norm)</t>
+  </si>
+  <si>
+    <t>Hasil</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,6 +84,14 @@
     <font>
       <sz val="11"/>
       <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -252,18 +270,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -276,35 +304,33 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -770,111 +796,111 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="E1" s="5" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="7"/>
-      <c r="I1" s="8"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="18"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>2.1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>-1.9</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>5.5</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>0.5</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <f>IF(A2&lt;=E2,0,1)</f>
         <v>1</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <f t="shared" ref="H2:I2" si="0">IF(B2&lt;=F2,0,1)</f>
         <v>0</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>-1.5</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>2.4</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>3.5</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <f>IF(A3&lt;=E2,0,1)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <f t="shared" ref="H3:I3" si="1">IF(B3&lt;=F2,0,1)</f>
         <v>1</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>0.5</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>-7.9</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>5.6</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <f>IF(A4&lt;=E2, 0,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <f t="shared" ref="H4:I4" si="2">IF(B4&lt;=F2, 0,1)</f>
         <v>0</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>5.9</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>-5.8</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <f>IF(A5&lt;=E2,0,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <f t="shared" ref="H5:I5" si="3">IF(B5&lt;=F2,0,1)</f>
         <v>1</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -899,336 +925,295 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
-      <c r="J1" s="9" t="s">
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="4"/>
+      <c r="J1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
       <c r="N1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>2.1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>-1.9</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>5.5</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="14"/>
-      <c r="H2" s="15"/>
-      <c r="J2" s="2">
+      <c r="G2" s="21"/>
+      <c r="H2" s="5"/>
+      <c r="J2" s="1">
         <v>2.1</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>-1.9</v>
       </c>
-      <c r="L2" s="2">
+      <c r="L2" s="1">
         <v>5.5</v>
       </c>
-      <c r="N2" s="24"/>
-      <c r="O2" s="4" t="s">
+      <c r="N2" s="13"/>
+      <c r="O2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="3"/>
+      <c r="P2" s="23"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>-1.5</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>2.4</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>3.5</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13">
+      <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3">
         <v>1</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="J3" s="2">
+      <c r="H3" s="5"/>
+      <c r="J3" s="1">
         <v>-1.5</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>2.4</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="1">
         <v>3.5</v>
       </c>
-      <c r="N3" s="25"/>
-      <c r="O3" s="21">
+      <c r="N3" s="14"/>
+      <c r="O3" s="11">
         <v>10</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>0.5</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>-7.9</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>5.6</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="15"/>
-      <c r="J4" s="2">
+      <c r="H4" s="5"/>
+      <c r="J4" s="1">
         <v>0.5</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>-7.9</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="1">
         <v>5.6</v>
       </c>
-      <c r="N4" s="23" t="s">
+      <c r="N4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="19">
         <f>MIN(O3:P3)</f>
         <v>10</v>
       </c>
-      <c r="P4" s="1"/>
+      <c r="P4" s="19"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>5.9</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>-5.8</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="15"/>
-      <c r="J5" s="2">
+      <c r="H5" s="5"/>
+      <c r="J5" s="1">
         <v>5.9</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>2.2999999999999998</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="1">
         <v>-5.8</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="19">
         <f>MAX(O3:P3)</f>
         <v>100</v>
       </c>
-      <c r="P5" s="1"/>
+      <c r="P5" s="19"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="16"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="15"/>
-      <c r="N6" s="20" t="s">
+      <c r="A6" s="6"/>
+      <c r="H6" s="5"/>
+      <c r="N6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="19">
         <f>O5-O4</f>
         <v>90</v>
       </c>
-      <c r="P6" s="1"/>
+      <c r="P6" s="19"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <f>MAX(A2:A5)</f>
         <v>5.9</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <f>MAX(B2:B5)</f>
         <v>2.4</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <f>MAX(C2:C5)</f>
         <v>5.6</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="15"/>
-      <c r="J7" s="2">
+      <c r="H7" s="5"/>
+      <c r="J7" s="1">
         <f>MAX(J2:J5)</f>
         <v>5.9</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <f t="shared" ref="K7:L7" si="0">MAX(K2:K5)</f>
         <v>2.4</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="1">
         <f t="shared" si="0"/>
         <v>5.6</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <f>MIN(A2:A5)</f>
         <v>-1.5</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="1">
         <f t="shared" ref="B8:C8" si="1">MIN(B2:B5)</f>
         <v>-7.9</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <f t="shared" si="1"/>
         <v>-5.8</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="15"/>
-      <c r="J8" s="2">
+      <c r="H8" s="5"/>
+      <c r="J8" s="1">
         <f>MIN(J2:J5)</f>
         <v>-1.5</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <f>MIN(K2:K5)</f>
         <v>-7.9</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="1">
         <f>MIN(L2:L5)</f>
         <v>-5.8</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="M8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <f>A7-A8</f>
         <v>7.4</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <f t="shared" ref="B9:C9" si="2">B7-B8</f>
         <v>10.3</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <f t="shared" si="2"/>
         <v>11.399999999999999</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="15"/>
-      <c r="J9" s="2">
+      <c r="H9" s="5"/>
+      <c r="J9" s="1">
         <f>J7-J8</f>
         <v>7.4</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <f t="shared" ref="K9:L9" si="3">K7-K8</f>
         <v>10.3</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="1">
         <f t="shared" si="3"/>
         <v>11.399999999999999</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="16"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="15"/>
+      <c r="A10" s="6"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A11" s="16">
+      <c r="A11" s="6">
         <f>(A2-A8)/(A9)</f>
         <v>0.48648648648648646</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11">
         <f t="shared" ref="B11:C11" si="4">(B2-B8)/(B9)</f>
         <v>0.58252427184466016</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11">
         <f t="shared" si="4"/>
         <v>0.99122807017543879</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="15"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A12" s="16">
+      <c r="A12" s="6">
         <f>(A3-A8)/A9</f>
         <v>0</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12">
         <f t="shared" ref="B12:C12" si="5">(B3-B8)/B9</f>
         <v>1</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12">
         <f t="shared" si="5"/>
         <v>0.81578947368421073</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="15"/>
+      <c r="H12" s="5"/>
       <c r="J12">
         <f>(((J2-J8)/J9)*O6)+O4</f>
         <v>53.783783783783782</v>
@@ -1243,23 +1228,19 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
+      <c r="A13" s="6">
         <f>(A4-A8)/A9</f>
         <v>0.27027027027027023</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13">
         <f t="shared" ref="B13:C13" si="6">(B4-B8)/B9</f>
         <v>0</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13">
         <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="15"/>
+      <c r="H13" s="5"/>
       <c r="J13">
         <f>(J3-J8)/J9*O6+O4</f>
         <v>10</v>
@@ -1274,23 +1255,19 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="16">
+      <c r="A14" s="6">
         <f>(A5-A8)/A9</f>
         <v>1</v>
       </c>
-      <c r="B14" s="13">
+      <c r="B14">
         <f t="shared" ref="B14:C14" si="7">(B5-B8)/B9</f>
         <v>0.99029126213592222</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="15"/>
+      <c r="H14" s="5"/>
       <c r="J14">
         <f>(J4-J8)/J9*O6+O4</f>
         <v>34.324324324324323</v>
@@ -1305,14 +1282,7 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="15"/>
+      <c r="H15" s="5"/>
       <c r="J15">
         <f>(J5-J8)/J9*O6+O4</f>
         <v>100</v>
@@ -1327,54 +1297,30 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="16"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="15"/>
+      <c r="A16" s="6"/>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="16"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="15"/>
+      <c r="A17" s="6"/>
+      <c r="H17" s="5"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="16"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="15"/>
+      <c r="A18" s="6"/>
+      <c r="H18" s="5"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="16"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="15"/>
+      <c r="A19" s="6"/>
+      <c r="H19" s="5"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1391,4 +1337,176 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97907AB2-8129-4F5B-A6BD-99FE6FC570D4}">
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="E4" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="I4" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="B5" s="1">
+        <v>-1.9</v>
+      </c>
+      <c r="C5" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="E5" s="25">
+        <f>ABS(A5) + ABS(B5) + ABS(C5)</f>
+        <v>9.5</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="I5" s="1">
+        <f>A5/$E$5</f>
+        <v>0.22105263157894739</v>
+      </c>
+      <c r="J5" s="1">
+        <f t="shared" ref="J5:K5" si="0">B5/$E$5</f>
+        <v>-0.19999999999999998</v>
+      </c>
+      <c r="K5" s="1">
+        <f t="shared" si="0"/>
+        <v>0.57894736842105265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>-1.5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2.4</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="E6" s="25">
+        <f t="shared" ref="E6:E8" si="1">ABS(A6) + ABS(B6) + ABS(C6)</f>
+        <v>7.4</v>
+      </c>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="I6" s="1">
+        <f>A6/$E$6</f>
+        <v>-0.20270270270270269</v>
+      </c>
+      <c r="J6" s="1">
+        <f t="shared" ref="J6:K6" si="2">B6/$E$6</f>
+        <v>0.32432432432432429</v>
+      </c>
+      <c r="K6" s="1">
+        <f t="shared" si="2"/>
+        <v>0.47297297297297297</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="B7" s="1">
+        <v>-7.9</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="E7" s="25">
+        <f>ABS(A7) + ABS(B7) + ABS(C7)</f>
+        <v>14</v>
+      </c>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="I7" s="1">
+        <f>A7/$E$7</f>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="J7" s="1">
+        <f t="shared" ref="J7:K7" si="3">B7/$E$7</f>
+        <v>-0.56428571428571428</v>
+      </c>
+      <c r="K7" s="1">
+        <f t="shared" si="3"/>
+        <v>0.39999999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C8" s="1">
+        <v>-5.8</v>
+      </c>
+      <c r="E8" s="25">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="I8" s="1">
+        <f>A8/$E$8</f>
+        <v>0.42142857142857143</v>
+      </c>
+      <c r="J8" s="1">
+        <f t="shared" ref="J8:K8" si="4">B8/$E$8</f>
+        <v>0.16428571428571428</v>
+      </c>
+      <c r="K8" s="1">
+        <f t="shared" si="4"/>
+        <v>-0.41428571428571426</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="E7:G7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
perhitungan manual dan otomatis di excel mengenai Least Squares
</commit_message>
<xml_diff>
--- a/Excel/004 Data Processing.xlsx
+++ b/Excel/004 Data Processing.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CD19F8-7A53-44C2-9894-5D56AD83F997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B19D1A3-CAFA-4BB5-A870-1F55B222ABCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Binarisation" sheetId="1" r:id="rId1"/>
     <sheet name="Scalling" sheetId="2" r:id="rId2"/>
     <sheet name="Normalisation (L1)" sheetId="3" r:id="rId3"/>
+    <sheet name="Normalisation (L2)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
   <si>
     <t>sample_data</t>
   </si>
@@ -61,12 +62,36 @@
   <si>
     <t>Hasil</t>
   </si>
+  <si>
+    <t>Least Squares</t>
+  </si>
+  <si>
+    <t>Jumlah Kuadrat</t>
+  </si>
+  <si>
+    <t>Perhitungan Manual Kuadrat</t>
+  </si>
+  <si>
+    <t>Akar (Jumlah Kuadrat)</t>
+  </si>
+  <si>
+    <t>Kuadrat</t>
+  </si>
+  <si>
+    <t>Hasil (Kuadrat / Akar)</t>
+  </si>
+  <si>
+    <t>Perhitungan Otomatis</t>
+  </si>
+  <si>
+    <t>Hasil Akhir</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +115,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="20"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -97,7 +130,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -107,6 +140,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -270,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -325,12 +382,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1348,20 +1442,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
@@ -1369,16 +1463,16 @@
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="I4" s="27" t="s">
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="I4" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
@@ -1509,4 +1603,327 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E53EC213-C428-409E-BAEC-B7450FDC2AC6}">
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="10" max="10" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="E3" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="O3" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="E4" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="33"/>
+      <c r="J4" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="O4" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="38">
+        <v>2.1</v>
+      </c>
+      <c r="B5" s="38">
+        <v>-1.9</v>
+      </c>
+      <c r="C5" s="38">
+        <v>5.5</v>
+      </c>
+      <c r="E5" s="34">
+        <f>A5^2</f>
+        <v>4.41</v>
+      </c>
+      <c r="F5" s="34">
+        <f>B5^2</f>
+        <v>3.61</v>
+      </c>
+      <c r="G5" s="34">
+        <f>C5^2</f>
+        <v>30.25</v>
+      </c>
+      <c r="H5" s="35">
+        <f>SUM(E5:G5)</f>
+        <v>38.269999999999996</v>
+      </c>
+      <c r="I5" s="41"/>
+      <c r="J5" s="42">
+        <f>SQRT(H5)</f>
+        <v>6.1862751312886166</v>
+      </c>
+      <c r="K5" s="38">
+        <f xml:space="preserve"> A5/J5</f>
+        <v>0.33946113863877969</v>
+      </c>
+      <c r="L5" s="38">
+        <f>B5/J5</f>
+        <v>-0.30713150638746733</v>
+      </c>
+      <c r="M5" s="38">
+        <f>C5/J5</f>
+        <v>0.88906488691108965</v>
+      </c>
+      <c r="O5" s="38">
+        <f>A5 / SQRT(SUMSQ(A5:C5))</f>
+        <v>0.33946113863877969</v>
+      </c>
+      <c r="P5" s="38">
+        <f>B5/(SQRT(SUMSQ(A5:C5)))</f>
+        <v>-0.30713150638746733</v>
+      </c>
+      <c r="Q5" s="38">
+        <f>C5 / SQRT(SUMSQ(A5:C5))</f>
+        <v>0.88906488691108965</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="38">
+        <v>-1.5</v>
+      </c>
+      <c r="B6" s="38">
+        <v>2.4</v>
+      </c>
+      <c r="C6" s="38">
+        <v>3.5</v>
+      </c>
+      <c r="E6" s="34">
+        <f>A6^2</f>
+        <v>2.25</v>
+      </c>
+      <c r="F6" s="34">
+        <f t="shared" ref="F6:F8" si="0">B6^2</f>
+        <v>5.76</v>
+      </c>
+      <c r="G6" s="34">
+        <f t="shared" ref="G6:G8" si="1">C6^2</f>
+        <v>12.25</v>
+      </c>
+      <c r="H6" s="35">
+        <f>SUM(E6:G6)</f>
+        <v>20.259999999999998</v>
+      </c>
+      <c r="I6" s="41"/>
+      <c r="J6" s="42">
+        <f t="shared" ref="J6:J8" si="2">SQRT(H6)</f>
+        <v>4.5011109739707598</v>
+      </c>
+      <c r="K6" s="38">
+        <f t="shared" ref="K6:K8" si="3" xml:space="preserve"> A6/J6</f>
+        <v>-0.33325105927720333</v>
+      </c>
+      <c r="L6" s="38">
+        <f t="shared" ref="L6:L8" si="4">B6/J6</f>
+        <v>0.53320169484352531</v>
+      </c>
+      <c r="M6" s="38">
+        <f t="shared" ref="M6:M8" si="5">C6/J6</f>
+        <v>0.77758580498014107</v>
+      </c>
+      <c r="O6" s="38">
+        <f t="shared" ref="O6:O8" si="6">A6 / SQRT(SUMSQ(A6:C6))</f>
+        <v>-0.33325105927720333</v>
+      </c>
+      <c r="P6" s="38">
+        <f t="shared" ref="P6:P8" si="7">B6/(SQRT(SUMSQ(A6:C6)))</f>
+        <v>0.53320169484352531</v>
+      </c>
+      <c r="Q6" s="38">
+        <f t="shared" ref="Q6:Q8" si="8">C6 / SQRT(SUMSQ(A6:C6))</f>
+        <v>0.77758580498014107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="38">
+        <v>0.5</v>
+      </c>
+      <c r="B7" s="38">
+        <v>-7.9</v>
+      </c>
+      <c r="C7" s="38">
+        <v>5.6</v>
+      </c>
+      <c r="E7" s="34">
+        <f t="shared" ref="E6:E8" si="9">A7^2</f>
+        <v>0.25</v>
+      </c>
+      <c r="F7" s="34">
+        <f t="shared" si="0"/>
+        <v>62.410000000000004</v>
+      </c>
+      <c r="G7" s="34">
+        <f t="shared" si="1"/>
+        <v>31.359999999999996</v>
+      </c>
+      <c r="H7" s="35">
+        <f>SUM(E7:G7)</f>
+        <v>94.02</v>
+      </c>
+      <c r="I7" s="41"/>
+      <c r="J7" s="42">
+        <f t="shared" si="2"/>
+        <v>9.6963910812219201</v>
+      </c>
+      <c r="K7" s="38">
+        <f t="shared" si="3"/>
+        <v>5.1565576905030421E-2</v>
+      </c>
+      <c r="L7" s="38">
+        <f t="shared" si="4"/>
+        <v>-0.81473611509948074</v>
+      </c>
+      <c r="M7" s="38">
+        <f t="shared" si="5"/>
+        <v>0.57753446133634068</v>
+      </c>
+      <c r="O7" s="38">
+        <f t="shared" si="6"/>
+        <v>5.1565576905030421E-2</v>
+      </c>
+      <c r="P7" s="38">
+        <f t="shared" si="7"/>
+        <v>-0.81473611509948074</v>
+      </c>
+      <c r="Q7" s="38">
+        <f t="shared" si="8"/>
+        <v>0.57753446133634068</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="38">
+        <v>5.9</v>
+      </c>
+      <c r="B8" s="38">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C8" s="38">
+        <v>-5.8</v>
+      </c>
+      <c r="E8" s="34">
+        <f t="shared" si="9"/>
+        <v>34.81</v>
+      </c>
+      <c r="F8" s="34">
+        <f t="shared" si="0"/>
+        <v>5.2899999999999991</v>
+      </c>
+      <c r="G8" s="34">
+        <f t="shared" si="1"/>
+        <v>33.64</v>
+      </c>
+      <c r="H8" s="35">
+        <f>SUM(E8:G8)</f>
+        <v>73.740000000000009</v>
+      </c>
+      <c r="I8" s="41"/>
+      <c r="J8" s="42">
+        <f t="shared" si="2"/>
+        <v>8.587199776411401</v>
+      </c>
+      <c r="K8" s="38">
+        <f t="shared" si="3"/>
+        <v>0.6870691440307467</v>
+      </c>
+      <c r="L8" s="38">
+        <f t="shared" si="4"/>
+        <v>0.26784051377469781</v>
+      </c>
+      <c r="M8" s="38">
+        <f t="shared" si="5"/>
+        <v>-0.67542390430141186</v>
+      </c>
+      <c r="O8" s="38">
+        <f t="shared" si="6"/>
+        <v>0.6870691440307467</v>
+      </c>
+      <c r="P8" s="38">
+        <f t="shared" si="7"/>
+        <v>0.26784051377469781</v>
+      </c>
+      <c r="Q8" s="38">
+        <f t="shared" si="8"/>
+        <v>-0.67542390430141186</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="P9" s="37"/>
+      <c r="Q9" s="37"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="P10" s="36"/>
+      <c r="Q10" s="36"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="E3:M3"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
perubahan sedikit pada hasil
</commit_message>
<xml_diff>
--- a/Excel/004 Data Processing.xlsx
+++ b/Excel/004 Data Processing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\006 Machine Learning\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B19D1A3-CAFA-4BB5-A870-1F55B222ABCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFDADDE-6437-44A5-8E2D-7C7DC6DA41DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,13 +78,13 @@
     <t>Kuadrat</t>
   </si>
   <si>
-    <t>Hasil (Kuadrat / Akar)</t>
-  </si>
-  <si>
     <t>Perhitungan Otomatis</t>
   </si>
   <si>
     <t>Hasil Akhir</t>
+  </si>
+  <si>
+    <t>Hasil (sample_data / Akar)</t>
   </si>
 </sst>
 </file>
@@ -1642,7 +1642,7 @@
       <c r="L3" s="39"/>
       <c r="M3" s="39"/>
       <c r="O3" s="40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P3" s="40"/>
       <c r="Q3" s="40"/>
@@ -1666,12 +1666,12 @@
         <v>14</v>
       </c>
       <c r="K4" s="28" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L4" s="28"/>
       <c r="M4" s="28"/>
       <c r="O4" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="P4" s="26"/>
       <c r="Q4" s="26"/>

</xml_diff>